<commit_message>
Address review: confirm request order, setUp evidence, run gap, tidy xlsx
</commit_message>
<xml_diff>
--- a/JMeter/JMeter-Results-35.xlsx
+++ b/JMeter/JMeter-Results-35.xlsx
@@ -10,10 +10,9 @@
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="TG1 per request" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Run checklist" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="TG2 per request" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="TG3 per request" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="TG4 per request" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="TG2 per request" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="TG3 per request" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="TG4 per request" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -59,12 +58,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="75">
   <si>
     <t xml:space="preserve">ParaBank JMeter results – Group 35 (Task 2)</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue = values typed from JMeter Aggregate Report TOTAL row. Yellow = still to fill after each run. Black = formulas.</t>
+    <t xml:space="preserve">Values typed from each JMeter Aggregate Report TOTAL row (blue). Black cells are formulas. Runs: 15 Oct 2026, each load run on its own with setUp.</t>
   </si>
   <si>
     <t xml:space="preserve">Metric</t>
@@ -184,7 +183,7 @@
     <t xml:space="preserve">TG1 – 1 user, Aggregate Report (GUI run, 15 Oct 2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">Typed from the Aggregate Report screenshot. Labels were cut off on screen, so request names assume rows appear in plan order – check against your screenshot after widening the Label column.</t>
+    <t xml:space="preserve">Typed from the Aggregate Report screenshot. JMeter lists rows in the order each request first runs, which matches the plan order (01 → 07).</t>
   </si>
   <si>
     <t xml:space="preserve">Label</t>
@@ -263,105 +262,6 @@
   </si>
   <si>
     <t xml:space="preserve">Percentiles (Median, 90/95/99%) cannot be recomputed from per-request rows, so the Summary uses JMeter's TOTAL row for those. Average uses the sample-weighted formula in C15.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidence checklist – per load</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Set Status with the dropdown. Wait 5–10 min between runs so Cloudflare's rate limit resets.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Load</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Step</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Save as</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aggregate Report screenshot (widen Label column first)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG1-aggregate.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">To do</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Save Table Data from Aggregate Report</t>
-  </si>
-  <si>
-    <t xml:space="preserve">results/TG1-aggregate.csv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">View Results Tree → 02 - Login → Request → Request Headers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG1-request-headers.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">View Results Tree → 02 - Login → Response data → Response headers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG1-response-headers.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG2-aggregate.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">results/TG2-aggregate.csv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG2-request-headers.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG2-response-headers.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG3-aggregate.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">results/TG3-aggregate.csv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG3-request-headers.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG3-response-headers.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG4-aggregate.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">results/TG4-aggregate.csv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG4-request-headers.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG4-response-headers.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Before each new load: enable that TG, disable the others, keep setUp enabled, click the broom (Clear All), then ▶.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Before committing: run  git checkout JMeter/jmeterplan-35.jmx  so the plan isn't committed with groups disabled.</t>
   </si>
   <si>
     <t xml:space="preserve">TG2 – 10 users, Aggregate Report (GUI run, 15 Oct 2026)</t>
@@ -1933,13 +1833,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="1" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1949,264 +1847,539 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="H3" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J3" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" s="18" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>73</v>
+      <c r="L3" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="M3" s="18" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>77</v>
+        <v>54</v>
+      </c>
+      <c r="B4" s="19" t="n">
+        <v>317</v>
+      </c>
+      <c r="C4" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="D4" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E4" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <v>28</v>
+      </c>
+      <c r="G4" s="19" t="n">
+        <v>239</v>
+      </c>
+      <c r="H4" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="I4" s="19" t="n">
+        <v>294</v>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>0.9621</v>
+      </c>
+      <c r="K4" s="13" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="L4" s="20" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="M4" s="20" t="n">
+        <v>2.15</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>77</v>
+        <v>55</v>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>317</v>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>27</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>199</v>
+      </c>
+      <c r="H5" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="I5" s="19" t="n">
+        <v>214</v>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>0.9653</v>
+      </c>
+      <c r="K5" s="13" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="L5" s="20" t="n">
+        <v>7.41</v>
+      </c>
+      <c r="M5" s="20" t="n">
+        <v>4.29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>77</v>
+        <v>56</v>
+      </c>
+      <c r="B6" s="19" t="n">
+        <v>316</v>
+      </c>
+      <c r="C6" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>195</v>
+      </c>
+      <c r="H6" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" s="19" t="n">
+        <v>236</v>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>0.9684</v>
+      </c>
+      <c r="K6" s="13" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="L6" s="20" t="n">
+        <v>10.44</v>
+      </c>
+      <c r="M6" s="20" t="n">
+        <v>2.28</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>77</v>
+        <v>57</v>
+      </c>
+      <c r="B7" s="19" t="n">
+        <v>316</v>
+      </c>
+      <c r="C7" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>19</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>192</v>
+      </c>
+      <c r="H7" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" s="19" t="n">
+        <v>197</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>0.9684</v>
+      </c>
+      <c r="K7" s="13" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="L7" s="20" t="n">
+        <v>7.59</v>
+      </c>
+      <c r="M7" s="20" t="n">
+        <v>3.49</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>77</v>
+        <v>58</v>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>315</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="I8" s="19" t="n">
+        <v>204</v>
+      </c>
+      <c r="J8" s="12" t="n">
+        <v>0.9714</v>
+      </c>
+      <c r="K8" s="13" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="L8" s="20" t="n">
+        <v>12.11</v>
+      </c>
+      <c r="M8" s="20" t="n">
+        <v>2.63</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>77</v>
+        <v>59</v>
+      </c>
+      <c r="B9" s="19" t="n">
+        <v>315</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>198</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" s="19" t="n">
+        <v>206</v>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>0.9714</v>
+      </c>
+      <c r="K9" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="L9" s="20" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="M9" s="20" t="n">
+        <v>3.7</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>77</v>
+        <v>60</v>
+      </c>
+      <c r="B10" s="19" t="n">
+        <v>315</v>
+      </c>
+      <c r="C10" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>19</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>199</v>
+      </c>
+      <c r="H10" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" s="19" t="n">
+        <v>216</v>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>0.9746</v>
+      </c>
+      <c r="K10" s="13" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="L10" s="20" t="n">
+        <v>11.18</v>
+      </c>
+      <c r="M10" s="20" t="n">
+        <v>2.38</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>77</v>
+        <v>61</v>
+      </c>
+      <c r="B11" s="19" t="n">
+        <v>315</v>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>195</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="I11" s="19" t="n">
+        <v>217</v>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>0.9778</v>
+      </c>
+      <c r="K11" s="13" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="L11" s="20" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="M11" s="20" t="n">
+        <v>5.18</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>77</v>
+        <v>62</v>
+      </c>
+      <c r="B12" s="19" t="n">
+        <v>315</v>
+      </c>
+      <c r="C12" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="D12" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>193</v>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="I12" s="19" t="n">
+        <v>345</v>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>0.9778</v>
+      </c>
+      <c r="K12" s="13" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="L12" s="20" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="M12" s="20" t="n">
+        <v>3.95</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>77</v>
+        <v>63</v>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>315</v>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>190</v>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" s="19" t="n">
+        <v>193</v>
+      </c>
+      <c r="J13" s="12" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="K13" s="13" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="L13" s="20" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="M13" s="20" t="n">
+        <v>2.42</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>77</v>
+      <c r="A14" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="22" t="n">
+        <v>3156</v>
+      </c>
+      <c r="C14" s="22" t="n">
+        <v>14</v>
+      </c>
+      <c r="D14" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="E14" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="F14" s="22" t="n">
+        <v>19</v>
+      </c>
+      <c r="G14" s="22" t="n">
+        <v>197</v>
+      </c>
+      <c r="H14" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="I14" s="22" t="n">
+        <v>345</v>
+      </c>
+      <c r="J14" s="23" t="n">
+        <v>0.9718</v>
+      </c>
+      <c r="K14" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="L14" s="22" t="n">
+        <v>86.94</v>
+      </c>
+      <c r="M14" s="22" t="n">
+        <v>30.73</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>77</v>
-      </c>
+      <c r="A15" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15" s="8" t="n">
+        <f aca="false">SUM(B4:B13)</f>
+        <v>3156</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <f aca="false">ROUND(SUMPRODUCT(B4:B13,C4:C13)/B15,0)</f>
+        <v>15</v>
+      </c>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8" t="n">
+        <f aca="false">MIN(H4:H13)</f>
+        <v>5</v>
+      </c>
+      <c r="I15" s="8" t="n">
+        <f aca="false">MAX(I4:I13)</f>
+        <v>345</v>
+      </c>
+      <c r="J15" s="11" t="n">
+        <f aca="false">SUMPRODUCT(B4:B13,J4:J13)/B15</f>
+        <v>0.971807541191382</v>
+      </c>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
-        <v>100</v>
+      <c r="A17" s="3" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4:D19" type="list">
-      <formula1>"Done,To do"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2231,7 +2404,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>101</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2271,7 +2444,7 @@
         <v>16</v>
       </c>
       <c r="K3" s="18" t="s">
-        <v>102</v>
+        <v>69</v>
       </c>
       <c r="L3" s="18" t="s">
         <v>52</v>
@@ -2285,40 +2458,40 @@
         <v>54</v>
       </c>
       <c r="B4" s="19" t="n">
-        <v>317</v>
+        <v>676</v>
       </c>
       <c r="C4" s="19" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G4" s="19" t="n">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="H4" s="19" t="n">
         <v>6</v>
       </c>
       <c r="I4" s="19" t="n">
-        <v>294</v>
+        <v>630</v>
       </c>
       <c r="J4" s="12" t="n">
-        <v>0.9621</v>
+        <v>0.9808</v>
       </c>
       <c r="K4" s="13" t="n">
-        <v>16.1</v>
+        <v>34.3</v>
       </c>
       <c r="L4" s="20" t="n">
-        <v>10.77</v>
+        <v>19.46</v>
       </c>
       <c r="M4" s="20" t="n">
-        <v>2.15</v>
+        <v>4.59</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2326,40 +2499,40 @@
         <v>55</v>
       </c>
       <c r="B5" s="19" t="n">
-        <v>317</v>
+        <v>676</v>
       </c>
       <c r="C5" s="19" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5" s="19" t="n">
         <v>9</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F5" s="19" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="G5" s="19" t="n">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H5" s="19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I5" s="19" t="n">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="J5" s="12" t="n">
-        <v>0.9653</v>
+        <v>0.9822</v>
       </c>
       <c r="K5" s="13" t="n">
-        <v>16.3</v>
+        <v>34.8</v>
       </c>
       <c r="L5" s="20" t="n">
-        <v>7.41</v>
+        <v>15.93</v>
       </c>
       <c r="M5" s="20" t="n">
-        <v>4.29</v>
+        <v>9.14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2367,40 +2540,40 @@
         <v>56</v>
       </c>
       <c r="B6" s="19" t="n">
-        <v>316</v>
+        <v>675</v>
       </c>
       <c r="C6" s="19" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D6" s="19" t="n">
         <v>9</v>
       </c>
       <c r="E6" s="19" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G6" s="19" t="n">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="H6" s="19" t="n">
         <v>5</v>
       </c>
       <c r="I6" s="19" t="n">
-        <v>236</v>
+        <v>216</v>
       </c>
       <c r="J6" s="12" t="n">
-        <v>0.9684</v>
+        <v>0.9837</v>
       </c>
       <c r="K6" s="13" t="n">
-        <v>16.4</v>
+        <v>35.1</v>
       </c>
       <c r="L6" s="20" t="n">
-        <v>10.44</v>
+        <v>19.35</v>
       </c>
       <c r="M6" s="20" t="n">
-        <v>2.28</v>
+        <v>4.84</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2408,40 +2581,40 @@
         <v>57</v>
       </c>
       <c r="B7" s="19" t="n">
-        <v>316</v>
+        <v>675</v>
       </c>
       <c r="C7" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E7" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="D7" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E7" s="19" t="n">
-        <v>12</v>
-      </c>
       <c r="F7" s="19" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G7" s="19" t="n">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="H7" s="19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I7" s="19" t="n">
-        <v>197</v>
+        <v>226</v>
       </c>
       <c r="J7" s="12" t="n">
-        <v>0.9684</v>
+        <v>0.9837</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>16.6</v>
+        <v>35.5</v>
       </c>
       <c r="L7" s="20" t="n">
-        <v>7.59</v>
+        <v>16.31</v>
       </c>
       <c r="M7" s="20" t="n">
-        <v>3.49</v>
+        <v>7.45</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2449,40 +2622,40 @@
         <v>58</v>
       </c>
       <c r="B8" s="19" t="n">
-        <v>315</v>
+        <v>675</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D8" s="19" t="n">
         <v>9</v>
       </c>
       <c r="E8" s="19" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="G8" s="19" t="n">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="H8" s="19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I8" s="19" t="n">
-        <v>204</v>
+        <v>220</v>
       </c>
       <c r="J8" s="12" t="n">
-        <v>0.9714</v>
+        <v>0.9837</v>
       </c>
       <c r="K8" s="13" t="n">
-        <v>16.8</v>
+        <v>35.9</v>
       </c>
       <c r="L8" s="20" t="n">
-        <v>12.11</v>
+        <v>21.82</v>
       </c>
       <c r="M8" s="20" t="n">
-        <v>2.63</v>
+        <v>5.56</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2490,40 +2663,40 @@
         <v>59</v>
       </c>
       <c r="B9" s="19" t="n">
-        <v>315</v>
+        <v>673</v>
       </c>
       <c r="C9" s="19" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D9" s="19" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F9" s="19" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="G9" s="19" t="n">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H9" s="19" t="n">
         <v>5</v>
       </c>
       <c r="I9" s="19" t="n">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="J9" s="12" t="n">
-        <v>0.9714</v>
+        <v>0.9866</v>
       </c>
       <c r="K9" s="13" t="n">
-        <v>17</v>
+        <v>36.3</v>
       </c>
       <c r="L9" s="20" t="n">
-        <v>7.76</v>
+        <v>16.66</v>
       </c>
       <c r="M9" s="20" t="n">
-        <v>3.7</v>
+        <v>7.87</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2531,40 +2704,40 @@
         <v>60</v>
       </c>
       <c r="B10" s="19" t="n">
-        <v>315</v>
+        <v>673</v>
       </c>
       <c r="C10" s="19" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D10" s="19" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E10" s="19" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G10" s="19" t="n">
         <v>199</v>
       </c>
       <c r="H10" s="19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I10" s="19" t="n">
         <v>216</v>
       </c>
       <c r="J10" s="12" t="n">
-        <v>0.9746</v>
+        <v>0.9866</v>
       </c>
       <c r="K10" s="13" t="n">
-        <v>17.2</v>
+        <v>36.7</v>
       </c>
       <c r="L10" s="20" t="n">
-        <v>11.18</v>
+        <v>20.58</v>
       </c>
       <c r="M10" s="20" t="n">
-        <v>2.38</v>
+        <v>5.05</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2572,40 +2745,40 @@
         <v>61</v>
       </c>
       <c r="B11" s="19" t="n">
-        <v>315</v>
+        <v>673</v>
       </c>
       <c r="C11" s="19" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D11" s="19" t="n">
         <v>9</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F11" s="19" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G11" s="19" t="n">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="H11" s="19" t="n">
         <v>6</v>
       </c>
       <c r="I11" s="19" t="n">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="J11" s="12" t="n">
-        <v>0.9778</v>
+        <v>0.9881</v>
       </c>
       <c r="K11" s="13" t="n">
-        <v>17.4</v>
+        <v>37.1</v>
       </c>
       <c r="L11" s="20" t="n">
-        <v>7.94</v>
+        <v>17.04</v>
       </c>
       <c r="M11" s="20" t="n">
-        <v>5.18</v>
+        <v>11.05</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2613,40 +2786,40 @@
         <v>62</v>
       </c>
       <c r="B12" s="19" t="n">
-        <v>315</v>
+        <v>673</v>
       </c>
       <c r="C12" s="19" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D12" s="19" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E12" s="19" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="H12" s="19" t="n">
         <v>5</v>
       </c>
       <c r="I12" s="19" t="n">
-        <v>345</v>
+        <v>224</v>
       </c>
       <c r="J12" s="12" t="n">
-        <v>0.9778</v>
+        <v>0.9896</v>
       </c>
       <c r="K12" s="13" t="n">
-        <v>17.6</v>
+        <v>37.5</v>
       </c>
       <c r="L12" s="20" t="n">
-        <v>8.23</v>
+        <v>17.45</v>
       </c>
       <c r="M12" s="20" t="n">
-        <v>3.95</v>
+        <v>8.43</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2654,40 +2827,40 @@
         <v>63</v>
       </c>
       <c r="B13" s="19" t="n">
-        <v>315</v>
+        <v>673</v>
       </c>
       <c r="C13" s="19" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D13" s="19" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>190</v>
+        <v>61</v>
       </c>
       <c r="H13" s="19" t="n">
         <v>6</v>
       </c>
       <c r="I13" s="19" t="n">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="J13" s="12" t="n">
-        <v>0.981</v>
+        <v>0.9896</v>
       </c>
       <c r="K13" s="13" t="n">
-        <v>17.7</v>
+        <v>38</v>
       </c>
       <c r="L13" s="20" t="n">
-        <v>8.15</v>
+        <v>17.47</v>
       </c>
       <c r="M13" s="20" t="n">
-        <v>2.42</v>
+        <v>5.15</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2695,40 +2868,40 @@
         <v>64</v>
       </c>
       <c r="B14" s="22" t="n">
-        <v>3156</v>
+        <v>6742</v>
       </c>
       <c r="C14" s="22" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D14" s="22" t="n">
         <v>9</v>
       </c>
       <c r="E14" s="22" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F14" s="22" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G14" s="22" t="n">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="H14" s="22" t="n">
         <v>5</v>
       </c>
       <c r="I14" s="22" t="n">
-        <v>345</v>
+        <v>630</v>
       </c>
       <c r="J14" s="23" t="n">
-        <v>0.9718</v>
+        <v>0.9855</v>
       </c>
       <c r="K14" s="22" t="s">
-        <v>103</v>
+        <v>72</v>
       </c>
       <c r="L14" s="22" t="n">
-        <v>86.94</v>
+        <v>172.64</v>
       </c>
       <c r="M14" s="22" t="n">
-        <v>30.73</v>
+        <v>65.37</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2737,11 +2910,11 @@
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">SUM(B4:B13)</f>
-        <v>3156</v>
+        <v>6742</v>
       </c>
       <c r="C15" s="8" t="n">
         <f aca="false">ROUND(SUMPRODUCT(B4:B13,C4:C13)/B15,0)</f>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
@@ -2753,11 +2926,11 @@
       </c>
       <c r="I15" s="8" t="n">
         <f aca="false">MAX(I4:I13)</f>
-        <v>345</v>
+        <v>630</v>
       </c>
       <c r="J15" s="11" t="n">
         <f aca="false">SUMPRODUCT(B4:B13,J4:J13)/B15</f>
-        <v>0.971807541191382</v>
+        <v>0.985454909522397</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8"/>
@@ -2793,7 +2966,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>104</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2833,7 +3006,7 @@
         <v>16</v>
       </c>
       <c r="K3" s="18" t="s">
-        <v>102</v>
+        <v>69</v>
       </c>
       <c r="L3" s="18" t="s">
         <v>52</v>
@@ -2847,40 +3020,40 @@
         <v>54</v>
       </c>
       <c r="B4" s="19" t="n">
-        <v>676</v>
+        <v>1680</v>
       </c>
       <c r="C4" s="19" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G4" s="19" t="n">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="H4" s="19" t="n">
         <v>6</v>
       </c>
       <c r="I4" s="19" t="n">
-        <v>630</v>
+        <v>616</v>
       </c>
       <c r="J4" s="12" t="n">
-        <v>0.9808</v>
+        <v>0.9905</v>
       </c>
       <c r="K4" s="13" t="n">
-        <v>34.3</v>
+        <v>85.3</v>
       </c>
       <c r="L4" s="20" t="n">
-        <v>19.46</v>
+        <v>43.82</v>
       </c>
       <c r="M4" s="20" t="n">
-        <v>4.59</v>
+        <v>11.42</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2888,40 +3061,40 @@
         <v>55</v>
       </c>
       <c r="B5" s="19" t="n">
-        <v>676</v>
+        <v>1680</v>
       </c>
       <c r="C5" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E5" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="D5" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E5" s="19" t="n">
-        <v>15</v>
-      </c>
       <c r="F5" s="19" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="G5" s="19" t="n">
-        <v>203</v>
+        <v>49</v>
       </c>
       <c r="H5" s="19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I5" s="19" t="n">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="J5" s="12" t="n">
-        <v>0.9822</v>
+        <v>0.9911</v>
       </c>
       <c r="K5" s="13" t="n">
-        <v>34.8</v>
+        <v>86.4</v>
       </c>
       <c r="L5" s="20" t="n">
-        <v>15.93</v>
+        <v>39.69</v>
       </c>
       <c r="M5" s="20" t="n">
-        <v>9.14</v>
+        <v>22.65</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2929,40 +3102,40 @@
         <v>56</v>
       </c>
       <c r="B6" s="19" t="n">
-        <v>675</v>
+        <v>1680</v>
       </c>
       <c r="C6" s="19" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6" s="19" t="n">
         <v>9</v>
       </c>
       <c r="E6" s="19" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G6" s="19" t="n">
-        <v>203</v>
+        <v>24</v>
       </c>
       <c r="H6" s="19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I6" s="19" t="n">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="J6" s="12" t="n">
-        <v>0.9837</v>
+        <v>0.9929</v>
       </c>
       <c r="K6" s="13" t="n">
-        <v>35.1</v>
+        <v>87.2</v>
       </c>
       <c r="L6" s="20" t="n">
-        <v>19.35</v>
+        <v>43.65</v>
       </c>
       <c r="M6" s="20" t="n">
-        <v>4.84</v>
+        <v>11.97</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2970,40 +3143,40 @@
         <v>57</v>
       </c>
       <c r="B7" s="19" t="n">
-        <v>675</v>
+        <v>1680</v>
       </c>
       <c r="C7" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E7" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="D7" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E7" s="19" t="n">
-        <v>15</v>
-      </c>
       <c r="F7" s="19" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G7" s="19" t="n">
-        <v>203</v>
+        <v>23</v>
       </c>
       <c r="H7" s="19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I7" s="19" t="n">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="J7" s="12" t="n">
-        <v>0.9837</v>
+        <v>0.9935</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>35.5</v>
+        <v>88.1</v>
       </c>
       <c r="L7" s="20" t="n">
-        <v>16.31</v>
+        <v>40.55</v>
       </c>
       <c r="M7" s="20" t="n">
-        <v>7.45</v>
+        <v>18.44</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3011,40 +3184,40 @@
         <v>58</v>
       </c>
       <c r="B8" s="19" t="n">
-        <v>675</v>
+        <v>1676</v>
       </c>
       <c r="C8" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E8" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="D8" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E8" s="19" t="n">
-        <v>15</v>
-      </c>
       <c r="F8" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="G8" s="19" t="n">
         <v>21</v>
       </c>
-      <c r="G8" s="19" t="n">
-        <v>203</v>
-      </c>
       <c r="H8" s="19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I8" s="19" t="n">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="J8" s="12" t="n">
-        <v>0.9837</v>
+        <v>0.994</v>
       </c>
       <c r="K8" s="13" t="n">
-        <v>35.9</v>
+        <v>88.8</v>
       </c>
       <c r="L8" s="20" t="n">
-        <v>21.82</v>
+        <v>45.71</v>
       </c>
       <c r="M8" s="20" t="n">
-        <v>5.56</v>
+        <v>13.73</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3052,40 +3225,40 @@
         <v>59</v>
       </c>
       <c r="B9" s="19" t="n">
-        <v>673</v>
+        <v>1671</v>
       </c>
       <c r="C9" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E9" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="D9" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E9" s="19" t="n">
-        <v>16</v>
-      </c>
       <c r="F9" s="19" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="G9" s="19" t="n">
-        <v>197</v>
+        <v>20</v>
       </c>
       <c r="H9" s="19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I9" s="19" t="n">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="J9" s="12" t="n">
-        <v>0.9866</v>
+        <v>0.9946</v>
       </c>
       <c r="K9" s="13" t="n">
-        <v>36.3</v>
+        <v>88.9</v>
       </c>
       <c r="L9" s="20" t="n">
-        <v>16.66</v>
+        <v>40.89</v>
       </c>
       <c r="M9" s="20" t="n">
-        <v>7.87</v>
+        <v>19.22</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3093,40 +3266,40 @@
         <v>60</v>
       </c>
       <c r="B10" s="19" t="n">
-        <v>673</v>
+        <v>1667</v>
       </c>
       <c r="C10" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="F10" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="D10" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E10" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="F10" s="19" t="n">
-        <v>20</v>
-      </c>
       <c r="G10" s="19" t="n">
-        <v>199</v>
+        <v>21</v>
       </c>
       <c r="H10" s="19" t="n">
         <v>6</v>
       </c>
       <c r="I10" s="19" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J10" s="12" t="n">
-        <v>0.9866</v>
+        <v>0.9952</v>
       </c>
       <c r="K10" s="13" t="n">
-        <v>36.7</v>
+        <v>90.1</v>
       </c>
       <c r="L10" s="20" t="n">
-        <v>20.58</v>
+        <v>44.76</v>
       </c>
       <c r="M10" s="20" t="n">
-        <v>5.05</v>
+        <v>12.36</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3134,40 +3307,40 @@
         <v>61</v>
       </c>
       <c r="B11" s="19" t="n">
-        <v>673</v>
+        <v>1663</v>
       </c>
       <c r="C11" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E11" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="D11" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E11" s="19" t="n">
-        <v>15</v>
-      </c>
       <c r="F11" s="19" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G11" s="19" t="n">
-        <v>201</v>
+        <v>20</v>
       </c>
       <c r="H11" s="19" t="n">
         <v>6</v>
       </c>
       <c r="I11" s="19" t="n">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="J11" s="12" t="n">
-        <v>0.9881</v>
+        <v>0.9958</v>
       </c>
       <c r="K11" s="13" t="n">
-        <v>37.1</v>
+        <v>90.9</v>
       </c>
       <c r="L11" s="20" t="n">
-        <v>17.04</v>
+        <v>41.85</v>
       </c>
       <c r="M11" s="20" t="n">
-        <v>11.05</v>
+        <v>27.03</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3175,40 +3348,40 @@
         <v>62</v>
       </c>
       <c r="B12" s="19" t="n">
-        <v>673</v>
+        <v>1659</v>
       </c>
       <c r="C12" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E12" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="D12" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E12" s="19" t="n">
-        <v>15</v>
-      </c>
       <c r="F12" s="19" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>195</v>
+        <v>21</v>
       </c>
       <c r="H12" s="19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I12" s="19" t="n">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="J12" s="12" t="n">
-        <v>0.9896</v>
+        <v>0.997</v>
       </c>
       <c r="K12" s="13" t="n">
-        <v>37.5</v>
+        <v>91.7</v>
       </c>
       <c r="L12" s="20" t="n">
-        <v>17.45</v>
+        <v>42.38</v>
       </c>
       <c r="M12" s="20" t="n">
-        <v>8.43</v>
+        <v>20.56</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3216,40 +3389,40 @@
         <v>63</v>
       </c>
       <c r="B13" s="19" t="n">
-        <v>673</v>
+        <v>1656</v>
       </c>
       <c r="C13" s="19" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D13" s="19" t="n">
         <v>9</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>61</v>
+        <v>16</v>
       </c>
       <c r="H13" s="19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I13" s="19" t="n">
-        <v>208</v>
+        <v>224</v>
       </c>
       <c r="J13" s="12" t="n">
-        <v>0.9896</v>
+        <v>0.9976</v>
       </c>
       <c r="K13" s="13" t="n">
-        <v>38</v>
+        <v>92.5</v>
       </c>
       <c r="L13" s="20" t="n">
-        <v>17.47</v>
+        <v>42.64</v>
       </c>
       <c r="M13" s="20" t="n">
-        <v>5.15</v>
+        <v>12.52</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3257,596 +3430,34 @@
         <v>64</v>
       </c>
       <c r="B14" s="22" t="n">
-        <v>6742</v>
+        <v>16712</v>
       </c>
       <c r="C14" s="22" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D14" s="22" t="n">
         <v>9</v>
       </c>
       <c r="E14" s="22" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F14" s="22" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="G14" s="22" t="n">
-        <v>202</v>
+        <v>45</v>
       </c>
       <c r="H14" s="22" t="n">
         <v>5</v>
       </c>
       <c r="I14" s="22" t="n">
-        <v>630</v>
-      </c>
-      <c r="J14" s="23" t="n">
-        <v>0.9855</v>
-      </c>
-      <c r="K14" s="22" t="s">
-        <v>105</v>
-      </c>
-      <c r="L14" s="22" t="n">
-        <v>172.64</v>
-      </c>
-      <c r="M14" s="22" t="n">
-        <v>65.37</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B15" s="8" t="n">
-        <f aca="false">SUM(B4:B13)</f>
-        <v>6742</v>
-      </c>
-      <c r="C15" s="8" t="n">
-        <f aca="false">ROUND(SUMPRODUCT(B4:B13,C4:C13)/B15,0)</f>
-        <v>13</v>
-      </c>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8" t="n">
-        <f aca="false">MIN(H4:H13)</f>
-        <v>5</v>
-      </c>
-      <c r="I15" s="8" t="n">
-        <f aca="false">MAX(I4:I13)</f>
-        <v>630</v>
-      </c>
-      <c r="J15" s="11" t="n">
-        <f aca="false">SUMPRODUCT(B4:B13,J4:J13)/B15</f>
-        <v>0.985454909522397</v>
-      </c>
-      <c r="K15" s="8"/>
-      <c r="L15" s="8"/>
-      <c r="M15" s="8"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:M17"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="1" width="12"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="E3" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="F3" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="G3" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="H3" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="I3" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="J3" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="K3" s="18" t="s">
-        <v>102</v>
-      </c>
-      <c r="L3" s="18" t="s">
-        <v>52</v>
-      </c>
-      <c r="M3" s="18" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B4" s="19" t="n">
-        <v>1680</v>
-      </c>
-      <c r="C4" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="D4" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E4" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="F4" s="19" t="n">
-        <v>28</v>
-      </c>
-      <c r="G4" s="19" t="n">
-        <v>195</v>
-      </c>
-      <c r="H4" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="I4" s="19" t="n">
-        <v>616</v>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>0.9905</v>
-      </c>
-      <c r="K4" s="13" t="n">
-        <v>85.3</v>
-      </c>
-      <c r="L4" s="20" t="n">
-        <v>43.82</v>
-      </c>
-      <c r="M4" s="20" t="n">
-        <v>11.42</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="B5" s="19" t="n">
-        <v>1680</v>
-      </c>
-      <c r="C5" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="D5" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E5" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="F5" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="G5" s="19" t="n">
-        <v>49</v>
-      </c>
-      <c r="H5" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="I5" s="19" t="n">
-        <v>218</v>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>0.9911</v>
-      </c>
-      <c r="K5" s="13" t="n">
-        <v>86.4</v>
-      </c>
-      <c r="L5" s="20" t="n">
-        <v>39.69</v>
-      </c>
-      <c r="M5" s="20" t="n">
-        <v>22.65</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" s="19" t="n">
-        <v>1680</v>
-      </c>
-      <c r="C6" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="D6" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E6" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="F6" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="G6" s="19" t="n">
-        <v>24</v>
-      </c>
-      <c r="H6" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="I6" s="19" t="n">
-        <v>218</v>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>0.9929</v>
-      </c>
-      <c r="K6" s="13" t="n">
-        <v>87.2</v>
-      </c>
-      <c r="L6" s="20" t="n">
-        <v>43.65</v>
-      </c>
-      <c r="M6" s="20" t="n">
-        <v>11.97</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B7" s="19" t="n">
-        <v>1680</v>
-      </c>
-      <c r="C7" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="D7" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E7" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="F7" s="19" t="n">
-        <v>17</v>
-      </c>
-      <c r="G7" s="19" t="n">
-        <v>23</v>
-      </c>
-      <c r="H7" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="I7" s="19" t="n">
-        <v>221</v>
-      </c>
-      <c r="J7" s="12" t="n">
-        <v>0.9935</v>
-      </c>
-      <c r="K7" s="13" t="n">
-        <v>88.1</v>
-      </c>
-      <c r="L7" s="20" t="n">
-        <v>40.55</v>
-      </c>
-      <c r="M7" s="20" t="n">
-        <v>18.44</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8" s="19" t="n">
-        <v>1676</v>
-      </c>
-      <c r="C8" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="D8" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E8" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="F8" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="G8" s="19" t="n">
-        <v>21</v>
-      </c>
-      <c r="H8" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="I8" s="19" t="n">
-        <v>212</v>
-      </c>
-      <c r="J8" s="12" t="n">
-        <v>0.994</v>
-      </c>
-      <c r="K8" s="13" t="n">
-        <v>88.8</v>
-      </c>
-      <c r="L8" s="20" t="n">
-        <v>45.71</v>
-      </c>
-      <c r="M8" s="20" t="n">
-        <v>13.73</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="B9" s="19" t="n">
-        <v>1671</v>
-      </c>
-      <c r="C9" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="D9" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E9" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="G9" s="19" t="n">
-        <v>20</v>
-      </c>
-      <c r="H9" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="I9" s="19" t="n">
-        <v>224</v>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>0.9946</v>
-      </c>
-      <c r="K9" s="13" t="n">
-        <v>88.9</v>
-      </c>
-      <c r="L9" s="20" t="n">
-        <v>40.89</v>
-      </c>
-      <c r="M9" s="20" t="n">
-        <v>19.22</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="B10" s="19" t="n">
-        <v>1667</v>
-      </c>
-      <c r="C10" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="D10" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E10" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="F10" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="G10" s="19" t="n">
-        <v>21</v>
-      </c>
-      <c r="H10" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="I10" s="19" t="n">
-        <v>215</v>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>0.9952</v>
-      </c>
-      <c r="K10" s="13" t="n">
-        <v>90.1</v>
-      </c>
-      <c r="L10" s="20" t="n">
-        <v>44.76</v>
-      </c>
-      <c r="M10" s="20" t="n">
-        <v>12.36</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="B11" s="19" t="n">
-        <v>1663</v>
-      </c>
-      <c r="C11" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="D11" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E11" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="F11" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="G11" s="19" t="n">
-        <v>20</v>
-      </c>
-      <c r="H11" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="I11" s="19" t="n">
-        <v>229</v>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>0.9958</v>
-      </c>
-      <c r="K11" s="13" t="n">
-        <v>90.9</v>
-      </c>
-      <c r="L11" s="20" t="n">
-        <v>41.85</v>
-      </c>
-      <c r="M11" s="20" t="n">
-        <v>27.03</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="B12" s="19" t="n">
-        <v>1659</v>
-      </c>
-      <c r="C12" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="D12" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E12" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="F12" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="G12" s="19" t="n">
-        <v>21</v>
-      </c>
-      <c r="H12" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="I12" s="19" t="n">
-        <v>225</v>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>0.997</v>
-      </c>
-      <c r="K12" s="13" t="n">
-        <v>91.7</v>
-      </c>
-      <c r="L12" s="20" t="n">
-        <v>42.38</v>
-      </c>
-      <c r="M12" s="20" t="n">
-        <v>20.56</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B13" s="19" t="n">
-        <v>1656</v>
-      </c>
-      <c r="C13" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="D13" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E13" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="F13" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="G13" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="H13" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>224</v>
-      </c>
-      <c r="J13" s="12" t="n">
-        <v>0.9976</v>
-      </c>
-      <c r="K13" s="13" t="n">
-        <v>92.5</v>
-      </c>
-      <c r="L13" s="20" t="n">
-        <v>42.64</v>
-      </c>
-      <c r="M13" s="20" t="n">
-        <v>12.52</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="B14" s="22" t="n">
-        <v>16712</v>
-      </c>
-      <c r="C14" s="22" t="n">
-        <v>11</v>
-      </c>
-      <c r="D14" s="22" t="n">
-        <v>9</v>
-      </c>
-      <c r="E14" s="22" t="n">
-        <v>12</v>
-      </c>
-      <c r="F14" s="22" t="n">
-        <v>14</v>
-      </c>
-      <c r="G14" s="22" t="n">
-        <v>45</v>
-      </c>
-      <c r="H14" s="22" t="n">
-        <v>5</v>
-      </c>
-      <c r="I14" s="22" t="n">
         <v>616</v>
       </c>
       <c r="J14" s="23" t="n">
         <v>0.9942</v>
       </c>
       <c r="K14" s="22" t="s">
-        <v>107</v>
+        <v>74</v>
       </c>
       <c r="L14" s="22" t="n">
         <v>403.53</v>

</xml_diff>